<commit_message>
Corrige valor da revisão
</commit_message>
<xml_diff>
--- a/valores_revisao.xlsx
+++ b/valores_revisao.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\yamaha-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931576D1-2F06-457E-BA52-BE4C2A9623CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E34F4CDE-C7A0-405D-A26B-BBEBFD43CE7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" xr2:uid="{834A019E-92C4-4C8B-8FB2-747C10F71E8A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{834A019E-92C4-4C8B-8FB2-747C10F71E8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -160,7 +160,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -168,14 +168,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -531,7 +530,7 @@
       <c r="D2" s="2">
         <v>6</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="3">
         <v>126</v>
       </c>
     </row>
@@ -548,7 +547,7 @@
       <c r="D3" s="2">
         <v>12</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="3">
         <v>126</v>
       </c>
     </row>
@@ -565,7 +564,7 @@
       <c r="D4" s="2">
         <v>18</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="3">
         <v>528</v>
       </c>
     </row>
@@ -582,7 +581,7 @@
       <c r="D5" s="2">
         <v>24</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="3">
         <v>330</v>
       </c>
     </row>
@@ -599,7 +598,7 @@
       <c r="D6" s="2">
         <v>30</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="3">
         <v>636</v>
       </c>
     </row>
@@ -616,7 +615,7 @@
       <c r="D7" s="2">
         <v>36</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="3">
         <v>414</v>
       </c>
     </row>
@@ -633,7 +632,7 @@
       <c r="D8" s="2">
         <v>42</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="3">
         <v>528</v>
       </c>
     </row>
@@ -650,7 +649,7 @@
       <c r="D9" s="2">
         <v>6</v>
       </c>
-      <c r="E9" s="6"/>
+      <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -665,7 +664,7 @@
       <c r="D10" s="2">
         <v>12</v>
       </c>
-      <c r="E10" s="6"/>
+      <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -680,7 +679,7 @@
       <c r="D11" s="2">
         <v>18</v>
       </c>
-      <c r="E11" s="6"/>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
@@ -695,7 +694,7 @@
       <c r="D12" s="2">
         <v>24</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -710,7 +709,7 @@
       <c r="D13" s="2">
         <v>30</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="4"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
@@ -725,7 +724,7 @@
       <c r="D14" s="2">
         <v>36</v>
       </c>
-      <c r="E14" s="6"/>
+      <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
@@ -740,7 +739,7 @@
       <c r="D15" s="2">
         <v>42</v>
       </c>
-      <c r="E15" s="6"/>
+      <c r="E15" s="4"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -755,7 +754,7 @@
       <c r="D16" s="2">
         <v>6</v>
       </c>
-      <c r="E16" s="6"/>
+      <c r="E16" s="4"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
@@ -770,7 +769,7 @@
       <c r="D17" s="2">
         <v>12</v>
       </c>
-      <c r="E17" s="3"/>
+      <c r="E17" s="4"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
@@ -785,7 +784,7 @@
       <c r="D18" s="2">
         <v>18</v>
       </c>
-      <c r="E18" s="3"/>
+      <c r="E18" s="4"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
@@ -800,7 +799,7 @@
       <c r="D19" s="2">
         <v>24</v>
       </c>
-      <c r="E19" s="3"/>
+      <c r="E19" s="4"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -815,7 +814,7 @@
       <c r="D20" s="2">
         <v>30</v>
       </c>
-      <c r="E20" s="3"/>
+      <c r="E20" s="4"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -830,7 +829,7 @@
       <c r="D21" s="2">
         <v>36</v>
       </c>
-      <c r="E21" s="3"/>
+      <c r="E21" s="4"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -845,7 +844,7 @@
       <c r="D22" s="2">
         <v>42</v>
       </c>
-      <c r="E22" s="3"/>
+      <c r="E22" s="4"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
@@ -860,7 +859,7 @@
       <c r="D23" s="2">
         <v>6</v>
       </c>
-      <c r="E23" s="3"/>
+      <c r="E23" s="4"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -875,7 +874,7 @@
       <c r="D24" s="2">
         <v>12</v>
       </c>
-      <c r="E24" s="3"/>
+      <c r="E24" s="4"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
@@ -890,7 +889,7 @@
       <c r="D25" s="2">
         <v>18</v>
       </c>
-      <c r="E25" s="3"/>
+      <c r="E25" s="4"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
@@ -905,7 +904,7 @@
       <c r="D26" s="2">
         <v>24</v>
       </c>
-      <c r="E26" s="3"/>
+      <c r="E26" s="4"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
@@ -920,7 +919,7 @@
       <c r="D27" s="2">
         <v>30</v>
       </c>
-      <c r="E27" s="3"/>
+      <c r="E27" s="4"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
@@ -935,7 +934,7 @@
       <c r="D28" s="2">
         <v>36</v>
       </c>
-      <c r="E28" s="3"/>
+      <c r="E28" s="4"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -950,7 +949,7 @@
       <c r="D29" s="2">
         <v>42</v>
       </c>
-      <c r="E29" s="3"/>
+      <c r="E29" s="4"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
@@ -965,7 +964,7 @@
       <c r="D30" s="2">
         <v>6</v>
       </c>
-      <c r="E30" s="4"/>
+      <c r="E30" s="5"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
@@ -980,7 +979,7 @@
       <c r="D31" s="2">
         <v>12</v>
       </c>
-      <c r="E31" s="4"/>
+      <c r="E31" s="5"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
@@ -995,7 +994,7 @@
       <c r="D32" s="2">
         <v>18</v>
       </c>
-      <c r="E32" s="4"/>
+      <c r="E32" s="5"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
@@ -1010,7 +1009,7 @@
       <c r="D33" s="2">
         <v>24</v>
       </c>
-      <c r="E33" s="4"/>
+      <c r="E33" s="5"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
@@ -1025,7 +1024,7 @@
       <c r="D34" s="2">
         <v>30</v>
       </c>
-      <c r="E34" s="3"/>
+      <c r="E34" s="4"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -1040,7 +1039,7 @@
       <c r="D35" s="2">
         <v>36</v>
       </c>
-      <c r="E35" s="3"/>
+      <c r="E35" s="4"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -1055,7 +1054,7 @@
       <c r="D36" s="2">
         <v>42</v>
       </c>
-      <c r="E36" s="3"/>
+      <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
@@ -1070,7 +1069,7 @@
       <c r="D37" s="2">
         <v>6</v>
       </c>
-      <c r="E37" s="3"/>
+      <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -1085,7 +1084,7 @@
       <c r="D38" s="2">
         <v>12</v>
       </c>
-      <c r="E38" s="3"/>
+      <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
@@ -1100,7 +1099,7 @@
       <c r="D39" s="2">
         <v>18</v>
       </c>
-      <c r="E39" s="3"/>
+      <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -1115,7 +1114,7 @@
       <c r="D40" s="2">
         <v>24</v>
       </c>
-      <c r="E40" s="3"/>
+      <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -1130,7 +1129,7 @@
       <c r="D41" s="2">
         <v>30</v>
       </c>
-      <c r="E41" s="3"/>
+      <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
@@ -1145,7 +1144,7 @@
       <c r="D42" s="2">
         <v>36</v>
       </c>
-      <c r="E42" s="3"/>
+      <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
@@ -1160,7 +1159,7 @@
       <c r="D43" s="2">
         <v>42</v>
       </c>
-      <c r="E43" s="3"/>
+      <c r="E43" s="4"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
@@ -1175,7 +1174,7 @@
       <c r="D44" s="2">
         <v>6</v>
       </c>
-      <c r="E44" s="3"/>
+      <c r="E44" s="4"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
@@ -1190,7 +1189,7 @@
       <c r="D45" s="2">
         <v>12</v>
       </c>
-      <c r="E45" s="3"/>
+      <c r="E45" s="4"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
@@ -1205,7 +1204,7 @@
       <c r="D46" s="2">
         <v>18</v>
       </c>
-      <c r="E46" s="3"/>
+      <c r="E46" s="4"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
@@ -1220,7 +1219,7 @@
       <c r="D47" s="2">
         <v>24</v>
       </c>
-      <c r="E47" s="3"/>
+      <c r="E47" s="4"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -1235,7 +1234,7 @@
       <c r="D48" s="2">
         <v>30</v>
       </c>
-      <c r="E48" s="3"/>
+      <c r="E48" s="4"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -1250,7 +1249,7 @@
       <c r="D49" s="2">
         <v>36</v>
       </c>
-      <c r="E49" s="3"/>
+      <c r="E49" s="4"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
@@ -1265,7 +1264,7 @@
       <c r="D50" s="2">
         <v>42</v>
       </c>
-      <c r="E50" s="3"/>
+      <c r="E50" s="4"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
@@ -1280,7 +1279,7 @@
       <c r="D51" s="2">
         <v>6</v>
       </c>
-      <c r="E51" s="3"/>
+      <c r="E51" s="4"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
@@ -1295,7 +1294,7 @@
       <c r="D52" s="2">
         <v>12</v>
       </c>
-      <c r="E52" s="3"/>
+      <c r="E52" s="4"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
@@ -1310,7 +1309,7 @@
       <c r="D53" s="2">
         <v>18</v>
       </c>
-      <c r="E53" s="3"/>
+      <c r="E53" s="4"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
@@ -1325,7 +1324,7 @@
       <c r="D54" s="2">
         <v>24</v>
       </c>
-      <c r="E54" s="3"/>
+      <c r="E54" s="4"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
@@ -1340,7 +1339,7 @@
       <c r="D55" s="2">
         <v>30</v>
       </c>
-      <c r="E55" s="3"/>
+      <c r="E55" s="4"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
@@ -1355,7 +1354,7 @@
       <c r="D56" s="2">
         <v>36</v>
       </c>
-      <c r="E56" s="3"/>
+      <c r="E56" s="4"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
@@ -1370,7 +1369,7 @@
       <c r="D57" s="2">
         <v>42</v>
       </c>
-      <c r="E57" s="3"/>
+      <c r="E57" s="4"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
@@ -1385,7 +1384,7 @@
       <c r="D58" s="2">
         <v>6</v>
       </c>
-      <c r="E58" s="3"/>
+      <c r="E58" s="4"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
@@ -1400,7 +1399,7 @@
       <c r="D59" s="2">
         <v>12</v>
       </c>
-      <c r="E59" s="3"/>
+      <c r="E59" s="4"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
@@ -1415,7 +1414,7 @@
       <c r="D60" s="2">
         <v>18</v>
       </c>
-      <c r="E60" s="3"/>
+      <c r="E60" s="4"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
@@ -1430,7 +1429,7 @@
       <c r="D61" s="2">
         <v>24</v>
       </c>
-      <c r="E61" s="3"/>
+      <c r="E61" s="4"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
@@ -1445,7 +1444,7 @@
       <c r="D62" s="2">
         <v>30</v>
       </c>
-      <c r="E62" s="3"/>
+      <c r="E62" s="4"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
@@ -1460,7 +1459,7 @@
       <c r="D63" s="2">
         <v>36</v>
       </c>
-      <c r="E63" s="3"/>
+      <c r="E63" s="4"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
@@ -1475,7 +1474,7 @@
       <c r="D64" s="2">
         <v>42</v>
       </c>
-      <c r="E64" s="3"/>
+      <c r="E64" s="4"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
@@ -1490,7 +1489,7 @@
       <c r="D65" s="2">
         <v>6</v>
       </c>
-      <c r="E65" s="3"/>
+      <c r="E65" s="4"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
@@ -1505,7 +1504,7 @@
       <c r="D66" s="2">
         <v>12</v>
       </c>
-      <c r="E66" s="3"/>
+      <c r="E66" s="4"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
@@ -1520,7 +1519,7 @@
       <c r="D67" s="2">
         <v>18</v>
       </c>
-      <c r="E67" s="3"/>
+      <c r="E67" s="4"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
@@ -1535,7 +1534,7 @@
       <c r="D68" s="2">
         <v>24</v>
       </c>
-      <c r="E68" s="3"/>
+      <c r="E68" s="4"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
@@ -1550,7 +1549,7 @@
       <c r="D69" s="2">
         <v>6</v>
       </c>
-      <c r="E69" s="3"/>
+      <c r="E69" s="4"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
@@ -1565,7 +1564,7 @@
       <c r="D70" s="2">
         <v>12</v>
       </c>
-      <c r="E70" s="3"/>
+      <c r="E70" s="4"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
@@ -1580,7 +1579,7 @@
       <c r="D71" s="2">
         <v>18</v>
       </c>
-      <c r="E71" s="3"/>
+      <c r="E71" s="4"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
@@ -1595,7 +1594,7 @@
       <c r="D72" s="2">
         <v>24</v>
       </c>
-      <c r="E72" s="3"/>
+      <c r="E72" s="4"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
@@ -1610,7 +1609,7 @@
       <c r="D73" s="2">
         <v>30</v>
       </c>
-      <c r="E73" s="3"/>
+      <c r="E73" s="4"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
@@ -1625,7 +1624,7 @@
       <c r="D74" s="2">
         <v>36</v>
       </c>
-      <c r="E74" s="3"/>
+      <c r="E74" s="4"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
@@ -1640,7 +1639,7 @@
       <c r="D75" s="2">
         <v>42</v>
       </c>
-      <c r="E75" s="3"/>
+      <c r="E75" s="4"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
@@ -1655,7 +1654,7 @@
       <c r="D76" s="2">
         <v>6</v>
       </c>
-      <c r="E76" s="3"/>
+      <c r="E76" s="4"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
@@ -1670,7 +1669,7 @@
       <c r="D77" s="2">
         <v>12</v>
       </c>
-      <c r="E77" s="3"/>
+      <c r="E77" s="4"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
@@ -1685,7 +1684,7 @@
       <c r="D78" s="2">
         <v>18</v>
       </c>
-      <c r="E78" s="3"/>
+      <c r="E78" s="4"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
@@ -1700,7 +1699,7 @@
       <c r="D79" s="2">
         <v>24</v>
       </c>
-      <c r="E79" s="3"/>
+      <c r="E79" s="4"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
@@ -1715,7 +1714,7 @@
       <c r="D80" s="2">
         <v>30</v>
       </c>
-      <c r="E80" s="3"/>
+      <c r="E80" s="4"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
@@ -1730,7 +1729,7 @@
       <c r="D81" s="2">
         <v>36</v>
       </c>
-      <c r="E81" s="3"/>
+      <c r="E81" s="4"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
@@ -1745,7 +1744,7 @@
       <c r="D82" s="2">
         <v>42</v>
       </c>
-      <c r="E82" s="3"/>
+      <c r="E82" s="4"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
@@ -1760,7 +1759,7 @@
       <c r="D83" s="2">
         <v>6</v>
       </c>
-      <c r="E83" s="3"/>
+      <c r="E83" s="4"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
@@ -1775,7 +1774,7 @@
       <c r="D84" s="2">
         <v>12</v>
       </c>
-      <c r="E84" s="3"/>
+      <c r="E84" s="4"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
@@ -1790,7 +1789,7 @@
       <c r="D85" s="2">
         <v>18</v>
       </c>
-      <c r="E85" s="3"/>
+      <c r="E85" s="4"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
@@ -1805,7 +1804,7 @@
       <c r="D86" s="2">
         <v>24</v>
       </c>
-      <c r="E86" s="3"/>
+      <c r="E86" s="4"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
@@ -1820,7 +1819,7 @@
       <c r="D87" s="2">
         <v>30</v>
       </c>
-      <c r="E87" s="3"/>
+      <c r="E87" s="4"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
@@ -1835,7 +1834,7 @@
       <c r="D88" s="2">
         <v>36</v>
       </c>
-      <c r="E88" s="3"/>
+      <c r="E88" s="4"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
@@ -1850,7 +1849,7 @@
       <c r="D89" s="2">
         <v>42</v>
       </c>
-      <c r="E89" s="3"/>
+      <c r="E89" s="4"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
@@ -1865,7 +1864,7 @@
       <c r="D90" s="2">
         <v>6</v>
       </c>
-      <c r="E90" s="3"/>
+      <c r="E90" s="4"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
@@ -1880,7 +1879,7 @@
       <c r="D91" s="2">
         <v>12</v>
       </c>
-      <c r="E91" s="3"/>
+      <c r="E91" s="4"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
@@ -1895,7 +1894,7 @@
       <c r="D92" s="2">
         <v>18</v>
       </c>
-      <c r="E92" s="3"/>
+      <c r="E92" s="4"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
@@ -1910,7 +1909,7 @@
       <c r="D93" s="2">
         <v>24</v>
       </c>
-      <c r="E93" s="3"/>
+      <c r="E93" s="4"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
@@ -1925,7 +1924,7 @@
       <c r="D94" s="2">
         <v>30</v>
       </c>
-      <c r="E94" s="3"/>
+      <c r="E94" s="4"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
@@ -1940,7 +1939,7 @@
       <c r="D95" s="2">
         <v>36</v>
       </c>
-      <c r="E95" s="3"/>
+      <c r="E95" s="4"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
@@ -1955,9 +1954,10 @@
       <c r="D96" s="2">
         <v>42</v>
       </c>
-      <c r="E96" s="3"/>
+      <c r="E96" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="172" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>